<commit_message>
Kalendarz: dodaj akademię 13.10 i rady szkoleniowe 21.10, 4.11, 18.11
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CJHQby44ceVKveQmrZKNz6
</commit_message>
<xml_diff>
--- a/kalendarz_dzienny_role_2026_2027.xlsx
+++ b/kalendarz_dzienny_role_2026_2027.xlsx
@@ -1489,7 +1489,11 @@
           <t>wtorek</t>
         </is>
       </c>
-      <c r="D44" s="3" t="n"/>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Dzień Nauczyciela – uroczysta akademia</t>
+        </is>
+      </c>
       <c r="E44" s="3" t="n"/>
       <c r="F44" s="3" t="n"/>
       <c r="G44" s="3" t="n"/>
@@ -1671,7 +1675,11 @@
       </c>
       <c r="D52" s="3" t="n"/>
       <c r="E52" s="3" t="n"/>
-      <c r="F52" s="3" t="n"/>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>15:45 - 18:45 - RADA PEDAGOGICZNA SZKOLENIOWA: praca z uczniem w spektrum autyzmu</t>
+        </is>
+      </c>
       <c r="G52" s="3" t="n"/>
       <c r="H52" s="6">
         <f>IF(A52&gt;DATE(2027,6,25),"",INT((A52-DATE(2026,8,31))/7)+1)</f>
@@ -1987,7 +1995,12 @@
       </c>
       <c r="D66" s="3" t="n"/>
       <c r="E66" s="3" t="n"/>
-      <c r="F66" s="3" t="n"/>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>15:45 - 17:45 - RADA PEDAGOGICZNA SZKOLENIOWA: platforma edukacyjna i narzędzia cyfrowe
+Szkolenie: korzystanie ze zintegrowanej platformy edukacyjnej i innych narzędzi cyfrowych w prowadzeniu lekcji (ok. 2 godziny)</t>
+        </is>
+      </c>
       <c r="G66" s="3" t="n"/>
       <c r="H66" s="6">
         <f>IF(A66&gt;DATE(2027,6,25),"",INT((A66-DATE(2026,8,31))/7)+1)</f>
@@ -2314,7 +2327,12 @@
         </is>
       </c>
       <c r="E80" s="3" t="n"/>
-      <c r="F80" s="3" t="n"/>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>15:45 - 18:45 - RADA PEDAGOGICZNA SZKOLENIOWA: uzależnienia cyfrowe (Fundacja Karan)
+Szkolenie Fundacji Karan: uzależnienia cyfrowe wśród młodzieży i nastolatków (ok. 3 godziny)</t>
+        </is>
+      </c>
       <c r="G80" s="3" t="n"/>
       <c r="H80" s="6">
         <f>IF(A80&gt;DATE(2027,6,25),"",INT((A80-DATE(2026,8,31))/7)+1)</f>

</xml_diff>

<commit_message>
Kalendarz: Dzień Nauczyciela 13.10 (akademia 16:00, kolacja 19:00) i praca nad dokumentacją 14.10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CJHQby44ceVKveQmrZKNz6
</commit_message>
<xml_diff>
--- a/kalendarz_dzienny_role_2026_2027.xlsx
+++ b/kalendarz_dzienny_role_2026_2027.xlsx
@@ -1491,11 +1491,17 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Dzień Nauczyciela – uroczysta akademia</t>
+          <t>16:00 - Uroczysta akademia z okazji Dnia Edukacji Narodowej
+Sala kinowa. Po akademii słodki poczęstunek.</t>
         </is>
       </c>
       <c r="E44" s="3" t="n"/>
-      <c r="F44" s="3" t="n"/>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>19:00 - Dzień Nauczyciela: uroczysta kolacja i zabawa taneczna
+Restauracja Impreza, ul. Morelowskiego 125A / Karmelkowa, Wrocław. Uroczysta kolacja, potem konkursy i wspólna zabawa taneczna. Potwierdź obecność na liście w pokoju nauczycielskim lub odpowiadając na wiadomość dyrektora.</t>
+        </is>
+      </c>
       <c r="G44" s="3" t="n"/>
       <c r="H44" s="6">
         <f>IF(A44&gt;DATE(2027,6,25),"",INT((A44-DATE(2026,8,31))/7)+1)</f>
@@ -1521,7 +1527,12 @@
         </is>
       </c>
       <c r="E45" s="3" t="n"/>
-      <c r="F45" s="3" t="n"/>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>Dzień bez zajęć dydaktycznych – nauczyciele do dyspozycji dyrektora
+Praca przy uzupełnianiu dokumentacji szkolnej, np. zaległe plany pracy, dane w dziennikach lekcyjnych (również nauczania indywidualnego), programy nauczania (zaktualizowane w wersji elektronicznej do p. dyr. Filusz), IPET-y, WOPFU itp.</t>
+        </is>
+      </c>
       <c r="G45" s="3" t="n"/>
       <c r="H45" s="6">
         <f>IF(A45&gt;DATE(2027,6,25),"",INT((A45-DATE(2026,8,31))/7)+1)</f>

</xml_diff>

<commit_message>
Kalendarz: matury próbne OKE 17–18.12.2026; aktualności: matury próbne i wyjście ucznia do toalety
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FwNciXjTxyxXV22TNGEse8
</commit_message>
<xml_diff>
--- a/kalendarz_dzienny_role_2026_2027.xlsx
+++ b/kalendarz_dzienny_role_2026_2027.xlsx
@@ -3124,8 +3124,18 @@
         </is>
       </c>
       <c r="D109" s="3" t="n"/>
-      <c r="E109" s="3" t="n"/>
-      <c r="F109" s="3" t="n"/>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>9:00 - MATURA PRÓBNA OKE: język polski
+Wychowawcy klas maturalnych i nauczyciele języka polskiego: proszę o przekazanie informacji uczniom. Matura próbna nie jest sprawdzeniem wiedzy na ocenę.</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>9:00 - MATURA PRÓBNA OKE: język polski
+Wychowawcy klas maturalnych i nauczyciele języka polskiego: proszę o przekazanie informacji uczniom. Matura próbna nie jest sprawdzeniem wiedzy na ocenę.</t>
+        </is>
+      </c>
       <c r="G109" s="3" t="n"/>
       <c r="H109" s="6">
         <f>IF(A109&gt;DATE(2027,6,25),"",INT((A109-DATE(2026,8,31))/7)+1)</f>
@@ -3146,8 +3156,18 @@
         </is>
       </c>
       <c r="D110" s="3" t="n"/>
-      <c r="E110" s="3" t="n"/>
-      <c r="F110" s="3" t="n"/>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>9:00 - MATURA PRÓBNA OKE: matematyka
+Wychowawcy klas maturalnych i nauczyciele matematyki: proszę o przekazanie informacji uczniom. Matura próbna nie jest sprawdzeniem wiedzy na ocenę.</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>9:00 - MATURA PRÓBNA OKE: matematyka
+Wychowawcy klas maturalnych i nauczyciele matematyki: proszę o przekazanie informacji uczniom. Matura próbna nie jest sprawdzeniem wiedzy na ocenę.</t>
+        </is>
+      </c>
       <c r="G110" s="3" t="n"/>
       <c r="H110" s="6">
         <f>IF(A110&gt;DATE(2027,6,25),"",INT((A110-DATE(2026,8,31))/7)+1)</f>

</xml_diff>

<commit_message>
Kalendarz: matury próbne OKE 17–18.12.2026; aktualności: matury próbne i wyjście ucznia do toalety (#34)
Claude-Session: https://claude.ai/code/session_01FwNciXjTxyxXV22TNGEse8

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/kalendarz_dzienny_role_2026_2027.xlsx
+++ b/kalendarz_dzienny_role_2026_2027.xlsx
@@ -3124,8 +3124,18 @@
         </is>
       </c>
       <c r="D109" s="3" t="n"/>
-      <c r="E109" s="3" t="n"/>
-      <c r="F109" s="3" t="n"/>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>9:00 - MATURA PRÓBNA OKE: język polski
+Wychowawcy klas maturalnych i nauczyciele języka polskiego: proszę o przekazanie informacji uczniom. Matura próbna nie jest sprawdzeniem wiedzy na ocenę.</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>9:00 - MATURA PRÓBNA OKE: język polski
+Wychowawcy klas maturalnych i nauczyciele języka polskiego: proszę o przekazanie informacji uczniom. Matura próbna nie jest sprawdzeniem wiedzy na ocenę.</t>
+        </is>
+      </c>
       <c r="G109" s="3" t="n"/>
       <c r="H109" s="6">
         <f>IF(A109&gt;DATE(2027,6,25),"",INT((A109-DATE(2026,8,31))/7)+1)</f>
@@ -3146,8 +3156,18 @@
         </is>
       </c>
       <c r="D110" s="3" t="n"/>
-      <c r="E110" s="3" t="n"/>
-      <c r="F110" s="3" t="n"/>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>9:00 - MATURA PRÓBNA OKE: matematyka
+Wychowawcy klas maturalnych i nauczyciele matematyki: proszę o przekazanie informacji uczniom. Matura próbna nie jest sprawdzeniem wiedzy na ocenę.</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>9:00 - MATURA PRÓBNA OKE: matematyka
+Wychowawcy klas maturalnych i nauczyciele matematyki: proszę o przekazanie informacji uczniom. Matura próbna nie jest sprawdzeniem wiedzy na ocenę.</t>
+        </is>
+      </c>
       <c r="G110" s="3" t="n"/>
       <c r="H110" s="6">
         <f>IF(A110&gt;DATE(2027,6,25),"",INT((A110-DATE(2026,8,31))/7)+1)</f>

</xml_diff>